<commit_message>
fix(tg-catalogo): dropdowns de Productos con rango util y _listas autoactualizable
El rango de Data Validation de Productos estaba fijo en la fila 72 mientras la
hoja ya tenia 100 filas: las ultimas 28 se cargaban sin desplegable y un material
tipeado con una tilde distinta dejaba al producto sin precio, sin ningun aviso.

- Productos: A2:A72/D2:D72 -> A2:A500/D2:D500.
- _listas dejaba de ser una lista estatica (tenia 11 materiales contra los 69 en
  uso) y pasa a 598 formulas matriciales CSE que leen los unicos de Materiales y
  Colecciones. Se descarto UNIQUE/spill: el archivo viaja entre LibreOffice y el
  Excel del cliente y el soporte no es parejo.
- fullCalcOnLoad para que recalcule al abrir.

Verificado abriendo en LibreOffice: aparecen los 73 materiales y 13 colecciones.
</commit_message>
<xml_diff>
--- a/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v3.xlsx
+++ b/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v3.xlsx
@@ -17,10 +17,10 @@
     <sheet name="_listas" sheetId="7" state="hidden" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="Colecciones_lista" vbProcedure="false">_listas!$B$2:$B$35</definedName>
-    <definedName function="false" hidden="false" name="Materiales_lista" vbProcedure="false">_listas!$A$2:$A$42</definedName>
+    <definedName function="false" hidden="false" name="Colecciones_lista" vbProcedure="false">_listas!$B$2:$B$500</definedName>
+    <definedName function="false" hidden="false" name="Materiales_lista" vbProcedure="false">_listas!$A$2:$A$500</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -5225,11 +5225,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" error="Elegí un material de la lista desplegable. Si necesitás uno nuevo, agregalo primero en la hoja Materiales." errorStyle="stop" errorTitle="Ese material no existe" operator="between" prompt="Elegí de la lista. Sale de la hoja Materiales." promptTitle="Material" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D2:D72" type="list">
+    <dataValidation allowBlank="true" error="Elegí un material de la lista desplegable. Si necesitás uno nuevo, agregalo primero en la hoja Materiales." errorStyle="stop" errorTitle="Ese material no existe" operator="between" prompt="Elegí de la lista. Sale de la hoja Materiales." promptTitle="Material" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D2:D500" type="list">
       <formula1>Materiales_lista</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Elegí una colección de la lista desplegable. Si necesitás una nueva, agregala primero en la hoja Colecciones." errorStyle="stop" errorTitle="Esa colección no existe" operator="between" prompt="Elegí de la lista. Sale de la hoja Colecciones." promptTitle="Colección" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A2:A72" type="list">
+    <dataValidation allowBlank="true" error="Elegí una colección de la lista desplegable. Si necesitás una nueva, agregala primero en la hoja Colecciones." errorStyle="stop" errorTitle="Esa colección no existe" operator="between" prompt="Elegí de la lista. Sale de la hoja Colecciones." promptTitle="Colección" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A2:A500" type="list">
       <formula1>Colecciones_lista</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -10174,7 +10174,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B300"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -10190,70 +10190,2395 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>93</v>
+      <c r="A2" s="8">
+        <f t="array" ref="A2">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A1,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B2" s="8">
+        <f t="array" ref="B2">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B1,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>95</v>
+      <c r="A3" s="8">
+        <f t="array" ref="A3">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A2,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B3" s="8">
+        <f t="array" ref="B3">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B2,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>97</v>
+      <c r="A4" s="8">
+        <f t="array" ref="A4">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A3,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B4" s="8">
+        <f t="array" ref="B4">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B3,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>99</v>
+      <c r="A5" s="8">
+        <f t="array" ref="A5">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A4,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B5" s="8">
+        <f t="array" ref="B5">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B4,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>169</v>
+      <c r="A6" s="8">
+        <f t="array" ref="A6">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A5,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B6" s="8">
+        <f t="array" ref="B6">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B5,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>118</v>
+      <c r="A7" s="8">
+        <f t="array" ref="A7">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A6,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B7" s="8">
+        <f t="array" ref="B7">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B6,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>155</v>
+      <c r="A8" s="8">
+        <f t="array" ref="A8">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A7,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B8" s="8">
+        <f t="array" ref="B8">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B7,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>142</v>
+      <c r="A9" s="8">
+        <f t="array" ref="A9">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A8,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B9" s="8">
+        <f t="array" ref="B9">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B8,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>171</v>
+      <c r="A10" s="8">
+        <f t="array" ref="A10">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A9,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B10" s="8">
+        <f t="array" ref="B10">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B9,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
-        <v>145</v>
+      <c r="A11" s="8">
+        <f t="array" ref="A11">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A10,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B11" s="8">
+        <f t="array" ref="B11">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B10,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
-        <v>134</v>
+      <c r="A12" s="8">
+        <f t="array" ref="A12">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A11,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B12" s="8">
+        <f t="array" ref="B12">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B11,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8">
+        <f t="array" ref="A13">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A12,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B13" s="8">
+        <f t="array" ref="B13">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B12,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8">
+        <f t="array" ref="A14">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A13,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B14" s="8">
+        <f t="array" ref="B14">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B13,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8">
+        <f t="array" ref="A15">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A14,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B15" s="8">
+        <f t="array" ref="B15">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B14,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8">
+        <f t="array" ref="A16">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A15,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B16" s="8">
+        <f t="array" ref="B16">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B15,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8">
+        <f t="array" ref="A17">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A16,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B17" s="8">
+        <f t="array" ref="B17">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B16,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8">
+        <f t="array" ref="A18">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A17,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B18" s="8">
+        <f t="array" ref="B18">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B17,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8">
+        <f t="array" ref="A19">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A18,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B19" s="8">
+        <f t="array" ref="B19">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B18,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8">
+        <f t="array" ref="A20">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A19,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B20" s="8">
+        <f t="array" ref="B20">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B19,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8">
+        <f t="array" ref="A21">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A20,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B21" s="8">
+        <f t="array" ref="B21">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B20,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8">
+        <f t="array" ref="A22">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A21,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B22" s="8">
+        <f t="array" ref="B22">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B21,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8">
+        <f t="array" ref="A23">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A22,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B23" s="8">
+        <f t="array" ref="B23">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B22,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8">
+        <f t="array" ref="A24">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A23,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B24" s="8">
+        <f t="array" ref="B24">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B23,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8">
+        <f t="array" ref="A25">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A24,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B25" s="8">
+        <f t="array" ref="B25">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B24,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8">
+        <f t="array" ref="A26">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A25,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B26" s="8">
+        <f t="array" ref="B26">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B25,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8">
+        <f t="array" ref="A27">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A26,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B27" s="8">
+        <f t="array" ref="B27">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B26,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8">
+        <f t="array" ref="A28">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A27,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B28" s="8">
+        <f t="array" ref="B28">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B27,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8">
+        <f t="array" ref="A29">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A28,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B29" s="8">
+        <f t="array" ref="B29">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B28,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8">
+        <f t="array" ref="A30">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A29,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B30" s="8">
+        <f t="array" ref="B30">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B29,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8">
+        <f t="array" ref="A31">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A30,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B31" s="8">
+        <f t="array" ref="B31">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B30,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8">
+        <f t="array" ref="A32">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A31,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B32" s="8">
+        <f t="array" ref="B32">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B31,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8">
+        <f t="array" ref="A33">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A32,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B33" s="8">
+        <f t="array" ref="B33">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B32,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8">
+        <f t="array" ref="A34">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A33,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B34" s="8">
+        <f t="array" ref="B34">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B33,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8">
+        <f t="array" ref="A35">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A34,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B35" s="8">
+        <f t="array" ref="B35">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B34,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8">
+        <f t="array" ref="A36">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A35,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B36" s="8">
+        <f t="array" ref="B36">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B35,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="8">
+        <f t="array" ref="A37">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A36,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B37" s="8">
+        <f t="array" ref="B37">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B36,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="8">
+        <f t="array" ref="A38">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A37,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B38" s="8">
+        <f t="array" ref="B38">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B37,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="8">
+        <f t="array" ref="A39">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A38,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B39" s="8">
+        <f t="array" ref="B39">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B38,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="8">
+        <f t="array" ref="A40">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A39,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B40" s="8">
+        <f t="array" ref="B40">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B39,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8">
+        <f t="array" ref="A41">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A40,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B41" s="8">
+        <f t="array" ref="B41">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B40,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="8">
+        <f t="array" ref="A42">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A41,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B42" s="8">
+        <f t="array" ref="B42">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B41,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="8">
+        <f t="array" ref="A43">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A42,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B43" s="8">
+        <f t="array" ref="B43">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B42,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="8">
+        <f t="array" ref="A44">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A43,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B44" s="8">
+        <f t="array" ref="B44">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B43,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="8">
+        <f t="array" ref="A45">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A44,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B45" s="8">
+        <f t="array" ref="B45">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B44,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="8">
+        <f t="array" ref="A46">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A45,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B46" s="8">
+        <f t="array" ref="B46">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B45,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="8">
+        <f t="array" ref="A47">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A46,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B47" s="8">
+        <f t="array" ref="B47">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B46,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="8">
+        <f t="array" ref="A48">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A47,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B48" s="8">
+        <f t="array" ref="B48">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B47,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="8">
+        <f t="array" ref="A49">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A48,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B49" s="8">
+        <f t="array" ref="B49">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B48,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="8">
+        <f t="array" ref="A50">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A49,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B50" s="8">
+        <f t="array" ref="B50">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B49,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="8">
+        <f t="array" ref="A51">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A50,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B51" s="8">
+        <f t="array" ref="B51">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B50,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="8">
+        <f t="array" ref="A52">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A51,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B52" s="8">
+        <f t="array" ref="B52">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B51,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="8">
+        <f t="array" ref="A53">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A52,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B53" s="8">
+        <f t="array" ref="B53">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B52,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="8">
+        <f t="array" ref="A54">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A53,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B54" s="8">
+        <f t="array" ref="B54">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B53,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="8">
+        <f t="array" ref="A55">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A54,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B55" s="8">
+        <f t="array" ref="B55">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B54,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="8">
+        <f t="array" ref="A56">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A55,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B56" s="8">
+        <f t="array" ref="B56">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B55,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="8">
+        <f t="array" ref="A57">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A56,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B57" s="8">
+        <f t="array" ref="B57">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B56,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="8">
+        <f t="array" ref="A58">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A57,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B58" s="8">
+        <f t="array" ref="B58">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B57,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="8">
+        <f t="array" ref="A59">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A58,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B59" s="8">
+        <f t="array" ref="B59">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B58,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="8">
+        <f t="array" ref="A60">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A59,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B60" s="8">
+        <f t="array" ref="B60">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B59,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="8">
+        <f t="array" ref="A61">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A60,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B61" s="8">
+        <f t="array" ref="B61">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B60,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="8">
+        <f t="array" ref="A62">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A61,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B62" s="8">
+        <f t="array" ref="B62">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B61,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="8">
+        <f t="array" ref="A63">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A62,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B63" s="8">
+        <f t="array" ref="B63">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B62,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="8">
+        <f t="array" ref="A64">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A63,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B64" s="8">
+        <f t="array" ref="B64">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B63,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="8">
+        <f t="array" ref="A65">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A64,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B65" s="8">
+        <f t="array" ref="B65">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B64,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="8">
+        <f t="array" ref="A66">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A65,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B66" s="8">
+        <f t="array" ref="B66">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B65,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="8">
+        <f t="array" ref="A67">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A66,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B67" s="8">
+        <f t="array" ref="B67">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B66,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="8">
+        <f t="array" ref="A68">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A67,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B68" s="8">
+        <f t="array" ref="B68">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B67,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="8">
+        <f t="array" ref="A69">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A68,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B69" s="8">
+        <f t="array" ref="B69">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B68,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="8">
+        <f t="array" ref="A70">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A69,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B70" s="8">
+        <f t="array" ref="B70">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B69,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="8">
+        <f t="array" ref="A71">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A70,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B71" s="8">
+        <f t="array" ref="B71">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B70,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="8">
+        <f t="array" ref="A72">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A71,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B72" s="8">
+        <f t="array" ref="B72">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B71,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="8">
+        <f t="array" ref="A73">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A72,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B73" s="8">
+        <f t="array" ref="B73">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B72,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="8">
+        <f t="array" ref="A74">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A73,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B74" s="8">
+        <f t="array" ref="B74">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B73,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="8">
+        <f t="array" ref="A75">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A74,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B75" s="8">
+        <f t="array" ref="B75">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B74,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="8">
+        <f t="array" ref="A76">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A75,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B76" s="8">
+        <f t="array" ref="B76">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B75,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="8">
+        <f t="array" ref="A77">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A76,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B77" s="8">
+        <f t="array" ref="B77">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B76,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="8">
+        <f t="array" ref="A78">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A77,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B78" s="8">
+        <f t="array" ref="B78">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B77,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="8">
+        <f t="array" ref="A79">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A78,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B79" s="8">
+        <f t="array" ref="B79">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B78,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="8">
+        <f t="array" ref="A80">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A79,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B80" s="8">
+        <f t="array" ref="B80">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B79,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="8">
+        <f t="array" ref="A81">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A80,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B81" s="8">
+        <f t="array" ref="B81">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B80,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="8">
+        <f t="array" ref="A82">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A81,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B82" s="8">
+        <f t="array" ref="B82">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B81,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="8">
+        <f t="array" ref="A83">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A82,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B83" s="8">
+        <f t="array" ref="B83">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B82,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="8">
+        <f t="array" ref="A84">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A83,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B84" s="8">
+        <f t="array" ref="B84">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B83,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="8">
+        <f t="array" ref="A85">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A84,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B85" s="8">
+        <f t="array" ref="B85">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B84,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="8">
+        <f t="array" ref="A86">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A85,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B86" s="8">
+        <f t="array" ref="B86">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B85,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="8">
+        <f t="array" ref="A87">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A86,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B87" s="8">
+        <f t="array" ref="B87">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B86,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="8">
+        <f t="array" ref="A88">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A87,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B88" s="8">
+        <f t="array" ref="B88">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B87,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="8">
+        <f t="array" ref="A89">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A88,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B89" s="8">
+        <f t="array" ref="B89">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B88,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="8">
+        <f t="array" ref="A90">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A89,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B90" s="8">
+        <f t="array" ref="B90">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B89,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="8">
+        <f t="array" ref="A91">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A90,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B91" s="8">
+        <f t="array" ref="B91">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B90,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="8">
+        <f t="array" ref="A92">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A91,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B92" s="8">
+        <f t="array" ref="B92">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B91,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="8">
+        <f t="array" ref="A93">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A92,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B93" s="8">
+        <f t="array" ref="B93">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B92,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="8">
+        <f t="array" ref="A94">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A93,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B94" s="8">
+        <f t="array" ref="B94">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B93,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="8">
+        <f t="array" ref="A95">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A94,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B95" s="8">
+        <f t="array" ref="B95">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B94,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="8">
+        <f t="array" ref="A96">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A95,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B96" s="8">
+        <f t="array" ref="B96">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B95,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="8">
+        <f t="array" ref="A97">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A96,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B97" s="8">
+        <f t="array" ref="B97">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B96,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="8">
+        <f t="array" ref="A98">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A97,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B98" s="8">
+        <f t="array" ref="B98">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B97,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="8">
+        <f t="array" ref="A99">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A98,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B99" s="8">
+        <f t="array" ref="B99">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B98,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="8">
+        <f t="array" ref="A100">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A99,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B100" s="8">
+        <f t="array" ref="B100">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B99,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="8">
+        <f t="array" ref="A101">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A100,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B101" s="8">
+        <f t="array" ref="B101">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B100,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="8">
+        <f t="array" ref="A102">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A101,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B102" s="8">
+        <f t="array" ref="B102">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B101,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="8">
+        <f t="array" ref="A103">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A102,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B103" s="8">
+        <f t="array" ref="B103">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B102,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="8">
+        <f t="array" ref="A104">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A103,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B104" s="8">
+        <f t="array" ref="B104">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B103,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="8">
+        <f t="array" ref="A105">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A104,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B105" s="8">
+        <f t="array" ref="B105">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B104,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="8">
+        <f t="array" ref="A106">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A105,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B106" s="8">
+        <f t="array" ref="B106">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B105,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="8">
+        <f t="array" ref="A107">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A106,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B107" s="8">
+        <f t="array" ref="B107">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B106,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="8">
+        <f t="array" ref="A108">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A107,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B108" s="8">
+        <f t="array" ref="B108">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B107,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="8">
+        <f t="array" ref="A109">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A108,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B109" s="8">
+        <f t="array" ref="B109">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B108,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="8">
+        <f t="array" ref="A110">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A109,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B110" s="8">
+        <f t="array" ref="B110">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B109,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="8">
+        <f t="array" ref="A111">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A110,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B111" s="8">
+        <f t="array" ref="B111">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B110,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="8">
+        <f t="array" ref="A112">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A111,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B112" s="8">
+        <f t="array" ref="B112">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B111,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="8">
+        <f t="array" ref="A113">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A112,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B113" s="8">
+        <f t="array" ref="B113">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B112,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="8">
+        <f t="array" ref="A114">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A113,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B114" s="8">
+        <f t="array" ref="B114">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B113,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="8">
+        <f t="array" ref="A115">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A114,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B115" s="8">
+        <f t="array" ref="B115">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B114,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="8">
+        <f t="array" ref="A116">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A115,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B116" s="8">
+        <f t="array" ref="B116">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B115,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="8">
+        <f t="array" ref="A117">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A116,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B117" s="8">
+        <f t="array" ref="B117">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B116,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="8">
+        <f t="array" ref="A118">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A117,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B118" s="8">
+        <f t="array" ref="B118">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B117,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="8">
+        <f t="array" ref="A119">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A118,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B119" s="8">
+        <f t="array" ref="B119">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B118,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="8">
+        <f t="array" ref="A120">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A119,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B120" s="8">
+        <f t="array" ref="B120">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B119,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="8">
+        <f t="array" ref="A121">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A120,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B121" s="8">
+        <f t="array" ref="B121">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B120,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="8">
+        <f t="array" ref="A122">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A121,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B122" s="8">
+        <f t="array" ref="B122">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B121,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="8">
+        <f t="array" ref="A123">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A122,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B123" s="8">
+        <f t="array" ref="B123">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B122,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="8">
+        <f t="array" ref="A124">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A123,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B124" s="8">
+        <f t="array" ref="B124">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B123,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="8">
+        <f t="array" ref="A125">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A124,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B125" s="8">
+        <f t="array" ref="B125">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B124,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="8">
+        <f t="array" ref="A126">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A125,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B126" s="8">
+        <f t="array" ref="B126">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B125,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="8">
+        <f t="array" ref="A127">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A126,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B127" s="8">
+        <f t="array" ref="B127">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B126,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="8">
+        <f t="array" ref="A128">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A127,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B128" s="8">
+        <f t="array" ref="B128">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B127,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="8">
+        <f t="array" ref="A129">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A128,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B129" s="8">
+        <f t="array" ref="B129">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B128,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="8">
+        <f t="array" ref="A130">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A129,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B130" s="8">
+        <f t="array" ref="B130">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B129,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="8">
+        <f t="array" ref="A131">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A130,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B131" s="8">
+        <f t="array" ref="B131">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B130,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="8">
+        <f t="array" ref="A132">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A131,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B132" s="8">
+        <f t="array" ref="B132">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B131,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="8">
+        <f t="array" ref="A133">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A132,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B133" s="8">
+        <f t="array" ref="B133">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B132,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="8">
+        <f t="array" ref="A134">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A133,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B134" s="8">
+        <f t="array" ref="B134">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B133,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="8">
+        <f t="array" ref="A135">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A134,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B135" s="8">
+        <f t="array" ref="B135">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B134,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="8">
+        <f t="array" ref="A136">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A135,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B136" s="8">
+        <f t="array" ref="B136">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B135,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="8">
+        <f t="array" ref="A137">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A136,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B137" s="8">
+        <f t="array" ref="B137">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B136,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="8">
+        <f t="array" ref="A138">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A137,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B138" s="8">
+        <f t="array" ref="B138">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B137,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="8">
+        <f t="array" ref="A139">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A138,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B139" s="8">
+        <f t="array" ref="B139">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B138,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="8">
+        <f t="array" ref="A140">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A139,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B140" s="8">
+        <f t="array" ref="B140">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B139,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="8">
+        <f t="array" ref="A141">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A140,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B141" s="8">
+        <f t="array" ref="B141">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B140,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="8">
+        <f t="array" ref="A142">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A141,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B142" s="8">
+        <f t="array" ref="B142">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B141,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="8">
+        <f t="array" ref="A143">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A142,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B143" s="8">
+        <f t="array" ref="B143">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B142,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="8">
+        <f t="array" ref="A144">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A143,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B144" s="8">
+        <f t="array" ref="B144">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B143,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="8">
+        <f t="array" ref="A145">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A144,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B145" s="8">
+        <f t="array" ref="B145">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B144,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="8">
+        <f t="array" ref="A146">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A145,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B146" s="8">
+        <f t="array" ref="B146">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B145,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="8">
+        <f t="array" ref="A147">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A146,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B147" s="8">
+        <f t="array" ref="B147">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B146,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="8">
+        <f t="array" ref="A148">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A147,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B148" s="8">
+        <f t="array" ref="B148">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B147,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="8">
+        <f t="array" ref="A149">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A148,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B149" s="8">
+        <f t="array" ref="B149">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B148,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="8">
+        <f t="array" ref="A150">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A149,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B150" s="8">
+        <f t="array" ref="B150">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B149,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="8">
+        <f t="array" ref="A151">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A150,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B151" s="8">
+        <f t="array" ref="B151">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B150,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="8">
+        <f t="array" ref="A152">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A151,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B152" s="8">
+        <f t="array" ref="B152">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B151,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="8">
+        <f t="array" ref="A153">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A152,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B153" s="8">
+        <f t="array" ref="B153">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B152,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="8">
+        <f t="array" ref="A154">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A153,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B154" s="8">
+        <f t="array" ref="B154">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B153,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="8">
+        <f t="array" ref="A155">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A154,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B155" s="8">
+        <f t="array" ref="B155">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B154,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="8">
+        <f t="array" ref="A156">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A155,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B156" s="8">
+        <f t="array" ref="B156">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B155,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="8">
+        <f t="array" ref="A157">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A156,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B157" s="8">
+        <f t="array" ref="B157">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B156,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="8">
+        <f t="array" ref="A158">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A157,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B158" s="8">
+        <f t="array" ref="B158">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B157,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="8">
+        <f t="array" ref="A159">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A158,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B159" s="8">
+        <f t="array" ref="B159">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B158,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="8">
+        <f t="array" ref="A160">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A159,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B160" s="8">
+        <f t="array" ref="B160">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B159,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="8">
+        <f t="array" ref="A161">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A160,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B161" s="8">
+        <f t="array" ref="B161">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B160,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="8">
+        <f t="array" ref="A162">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A161,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B162" s="8">
+        <f t="array" ref="B162">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B161,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="8">
+        <f t="array" ref="A163">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A162,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B163" s="8">
+        <f t="array" ref="B163">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B162,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="8">
+        <f t="array" ref="A164">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A163,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B164" s="8">
+        <f t="array" ref="B164">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B163,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="8">
+        <f t="array" ref="A165">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A164,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B165" s="8">
+        <f t="array" ref="B165">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B164,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="8">
+        <f t="array" ref="A166">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A165,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B166" s="8">
+        <f t="array" ref="B166">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B165,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="8">
+        <f t="array" ref="A167">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A166,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B167" s="8">
+        <f t="array" ref="B167">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B166,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="8">
+        <f t="array" ref="A168">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A167,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B168" s="8">
+        <f t="array" ref="B168">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B167,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="8">
+        <f t="array" ref="A169">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A168,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B169" s="8">
+        <f t="array" ref="B169">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B168,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="8">
+        <f t="array" ref="A170">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A169,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B170" s="8">
+        <f t="array" ref="B170">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B169,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="8">
+        <f t="array" ref="A171">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A170,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B171" s="8">
+        <f t="array" ref="B171">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B170,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="8">
+        <f t="array" ref="A172">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A171,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B172" s="8">
+        <f t="array" ref="B172">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B171,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="8">
+        <f t="array" ref="A173">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A172,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B173" s="8">
+        <f t="array" ref="B173">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B172,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="8">
+        <f t="array" ref="A174">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A173,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B174" s="8">
+        <f t="array" ref="B174">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B173,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="8">
+        <f t="array" ref="A175">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A174,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B175" s="8">
+        <f t="array" ref="B175">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B174,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="8">
+        <f t="array" ref="A176">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A175,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B176" s="8">
+        <f t="array" ref="B176">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B175,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="8">
+        <f t="array" ref="A177">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A176,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B177" s="8">
+        <f t="array" ref="B177">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B176,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="8">
+        <f t="array" ref="A178">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A177,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B178" s="8">
+        <f t="array" ref="B178">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B177,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="8">
+        <f t="array" ref="A179">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A178,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B179" s="8">
+        <f t="array" ref="B179">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B178,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="8">
+        <f t="array" ref="A180">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A179,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B180" s="8">
+        <f t="array" ref="B180">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B179,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="8">
+        <f t="array" ref="A181">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A180,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B181" s="8">
+        <f t="array" ref="B181">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B180,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="8">
+        <f t="array" ref="A182">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A181,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B182" s="8">
+        <f t="array" ref="B182">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B181,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="8">
+        <f t="array" ref="A183">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A182,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B183" s="8">
+        <f t="array" ref="B183">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B182,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="8">
+        <f t="array" ref="A184">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A183,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B184" s="8">
+        <f t="array" ref="B184">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B183,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="8">
+        <f t="array" ref="A185">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A184,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B185" s="8">
+        <f t="array" ref="B185">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B184,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="8">
+        <f t="array" ref="A186">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A185,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B186" s="8">
+        <f t="array" ref="B186">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B185,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="8">
+        <f t="array" ref="A187">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A186,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B187" s="8">
+        <f t="array" ref="B187">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B186,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="8">
+        <f t="array" ref="A188">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A187,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B188" s="8">
+        <f t="array" ref="B188">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B187,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="8">
+        <f t="array" ref="A189">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A188,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B189" s="8">
+        <f t="array" ref="B189">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B188,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="8">
+        <f t="array" ref="A190">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A189,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B190" s="8">
+        <f t="array" ref="B190">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B189,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="8">
+        <f t="array" ref="A191">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A190,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B191" s="8">
+        <f t="array" ref="B191">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B190,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="8">
+        <f t="array" ref="A192">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A191,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B192" s="8">
+        <f t="array" ref="B192">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B191,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A193" s="8">
+        <f t="array" ref="A193">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A192,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B193" s="8">
+        <f t="array" ref="B193">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B192,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="8">
+        <f t="array" ref="A194">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A193,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B194" s="8">
+        <f t="array" ref="B194">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B193,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A195" s="8">
+        <f t="array" ref="A195">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A194,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B195" s="8">
+        <f t="array" ref="B195">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B194,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="8">
+        <f t="array" ref="A196">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A195,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B196" s="8">
+        <f t="array" ref="B196">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B195,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="8">
+        <f t="array" ref="A197">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A196,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B197" s="8">
+        <f t="array" ref="B197">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B196,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="8">
+        <f t="array" ref="A198">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A197,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B198" s="8">
+        <f t="array" ref="B198">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B197,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="8">
+        <f t="array" ref="A199">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A198,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B199" s="8">
+        <f t="array" ref="B199">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B198,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="8">
+        <f t="array" ref="A200">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A199,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B200" s="8">
+        <f t="array" ref="B200">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B199,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="8">
+        <f t="array" ref="A201">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A200,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B201" s="8">
+        <f t="array" ref="B201">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B200,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="8">
+        <f t="array" ref="A202">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A201,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B202" s="8">
+        <f t="array" ref="B202">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B201,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="203" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="8">
+        <f t="array" ref="A203">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A202,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B203" s="8">
+        <f t="array" ref="B203">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B202,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="8">
+        <f t="array" ref="A204">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A203,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B204" s="8">
+        <f t="array" ref="B204">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B203,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="8">
+        <f t="array" ref="A205">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A204,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B205" s="8">
+        <f t="array" ref="B205">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B204,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="8">
+        <f t="array" ref="A206">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A205,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B206" s="8">
+        <f t="array" ref="B206">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B205,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A207" s="8">
+        <f t="array" ref="A207">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A206,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B207" s="8">
+        <f t="array" ref="B207">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B206,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A208" s="8">
+        <f t="array" ref="A208">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A207,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B208" s="8">
+        <f t="array" ref="B208">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B207,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A209" s="8">
+        <f t="array" ref="A209">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A208,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B209" s="8">
+        <f t="array" ref="B209">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B208,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A210" s="8">
+        <f t="array" ref="A210">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A209,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B210" s="8">
+        <f t="array" ref="B210">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B209,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A211" s="8">
+        <f t="array" ref="A211">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A210,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B211" s="8">
+        <f t="array" ref="B211">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B210,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A212" s="8">
+        <f t="array" ref="A212">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A211,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B212" s="8">
+        <f t="array" ref="B212">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B211,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="8">
+        <f t="array" ref="A213">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A212,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B213" s="8">
+        <f t="array" ref="B213">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B212,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="8">
+        <f t="array" ref="A214">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A213,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B214" s="8">
+        <f t="array" ref="B214">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B213,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="8">
+        <f t="array" ref="A215">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A214,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B215" s="8">
+        <f t="array" ref="B215">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B214,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="8">
+        <f t="array" ref="A216">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A215,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B216" s="8">
+        <f t="array" ref="B216">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B215,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="8">
+        <f t="array" ref="A217">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A216,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B217" s="8">
+        <f t="array" ref="B217">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B216,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="8">
+        <f t="array" ref="A218">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A217,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B218" s="8">
+        <f t="array" ref="B218">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B217,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="8">
+        <f t="array" ref="A219">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A218,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B219" s="8">
+        <f t="array" ref="B219">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B218,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="8">
+        <f t="array" ref="A220">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A219,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B220" s="8">
+        <f t="array" ref="B220">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B219,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="8">
+        <f t="array" ref="A221">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A220,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B221" s="8">
+        <f t="array" ref="B221">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B220,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="8">
+        <f t="array" ref="A222">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A221,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B222" s="8">
+        <f t="array" ref="B222">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B221,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="8">
+        <f t="array" ref="A223">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A222,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B223" s="8">
+        <f t="array" ref="B223">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B222,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="8">
+        <f t="array" ref="A224">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A223,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B224" s="8">
+        <f t="array" ref="B224">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B223,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="8">
+        <f t="array" ref="A225">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A224,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B225" s="8">
+        <f t="array" ref="B225">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B224,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="8">
+        <f t="array" ref="A226">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A225,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B226" s="8">
+        <f t="array" ref="B226">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B225,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="8">
+        <f t="array" ref="A227">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A226,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B227" s="8">
+        <f t="array" ref="B227">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B226,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="8">
+        <f t="array" ref="A228">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A227,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B228" s="8">
+        <f t="array" ref="B228">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B227,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="8">
+        <f t="array" ref="A229">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A228,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B229" s="8">
+        <f t="array" ref="B229">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B228,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="8">
+        <f t="array" ref="A230">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A229,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B230" s="8">
+        <f t="array" ref="B230">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B229,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="8">
+        <f t="array" ref="A231">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A230,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B231" s="8">
+        <f t="array" ref="B231">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B230,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="8">
+        <f t="array" ref="A232">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A231,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B232" s="8">
+        <f t="array" ref="B232">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B231,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="8">
+        <f t="array" ref="A233">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A232,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B233" s="8">
+        <f t="array" ref="B233">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B232,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="8">
+        <f t="array" ref="A234">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A233,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B234" s="8">
+        <f t="array" ref="B234">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B233,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="8">
+        <f t="array" ref="A235">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A234,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B235" s="8">
+        <f t="array" ref="B235">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B234,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="8">
+        <f t="array" ref="A236">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A235,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B236" s="8">
+        <f t="array" ref="B236">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B235,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="8">
+        <f t="array" ref="A237">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A236,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B237" s="8">
+        <f t="array" ref="B237">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B236,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A238" s="8">
+        <f t="array" ref="A238">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A237,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B238" s="8">
+        <f t="array" ref="B238">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B237,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A239" s="8">
+        <f t="array" ref="A239">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A238,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B239" s="8">
+        <f t="array" ref="B239">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B238,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A240" s="8">
+        <f t="array" ref="A240">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A239,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B240" s="8">
+        <f t="array" ref="B240">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B239,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A241" s="8">
+        <f t="array" ref="A241">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A240,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B241" s="8">
+        <f t="array" ref="B241">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B240,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A242" s="8">
+        <f t="array" ref="A242">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A241,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B242" s="8">
+        <f t="array" ref="B242">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B241,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="243" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="8">
+        <f t="array" ref="A243">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A242,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B243" s="8">
+        <f t="array" ref="B243">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B242,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="244" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A244" s="8">
+        <f t="array" ref="A244">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A243,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B244" s="8">
+        <f t="array" ref="B244">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B243,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A245" s="8">
+        <f t="array" ref="A245">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A244,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B245" s="8">
+        <f t="array" ref="B245">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B244,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="246" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A246" s="8">
+        <f t="array" ref="A246">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A245,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B246" s="8">
+        <f t="array" ref="B246">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B245,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A247" s="8">
+        <f t="array" ref="A247">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A246,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B247" s="8">
+        <f t="array" ref="B247">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B246,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="248" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="8">
+        <f t="array" ref="A248">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A247,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B248" s="8">
+        <f t="array" ref="B248">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B247,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="249" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A249" s="8">
+        <f t="array" ref="A249">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A248,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B249" s="8">
+        <f t="array" ref="B249">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B248,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="250" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A250" s="8">
+        <f t="array" ref="A250">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A249,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B250" s="8">
+        <f t="array" ref="B250">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B249,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="251" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A251" s="8">
+        <f t="array" ref="A251">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A250,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B251" s="8">
+        <f t="array" ref="B251">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B250,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="252" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A252" s="8">
+        <f t="array" ref="A252">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A251,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B252" s="8">
+        <f t="array" ref="B252">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B251,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A253" s="8">
+        <f t="array" ref="A253">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A252,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B253" s="8">
+        <f t="array" ref="B253">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B252,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="254" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A254" s="8">
+        <f t="array" ref="A254">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A253,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B254" s="8">
+        <f t="array" ref="B254">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B253,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="255" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A255" s="8">
+        <f t="array" ref="A255">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A254,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B255" s="8">
+        <f t="array" ref="B255">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B254,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A256" s="8">
+        <f t="array" ref="A256">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A255,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B256" s="8">
+        <f t="array" ref="B256">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B255,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="257" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A257" s="8">
+        <f t="array" ref="A257">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A256,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B257" s="8">
+        <f t="array" ref="B257">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B256,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A258" s="8">
+        <f t="array" ref="A258">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A257,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B258" s="8">
+        <f t="array" ref="B258">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B257,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="259" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A259" s="8">
+        <f t="array" ref="A259">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A258,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B259" s="8">
+        <f t="array" ref="B259">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B258,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="260" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="8">
+        <f t="array" ref="A260">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A259,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B260" s="8">
+        <f t="array" ref="B260">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B259,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="261" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="8">
+        <f t="array" ref="A261">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A260,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B261" s="8">
+        <f t="array" ref="B261">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B260,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A262" s="8">
+        <f t="array" ref="A262">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A261,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B262" s="8">
+        <f t="array" ref="B262">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B261,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="263" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A263" s="8">
+        <f t="array" ref="A263">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A262,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B263" s="8">
+        <f t="array" ref="B263">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B262,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="264" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A264" s="8">
+        <f t="array" ref="A264">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A263,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B264" s="8">
+        <f t="array" ref="B264">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B263,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="265" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A265" s="8">
+        <f t="array" ref="A265">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A264,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B265" s="8">
+        <f t="array" ref="B265">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B264,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="266" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="8">
+        <f t="array" ref="A266">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A265,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B266" s="8">
+        <f t="array" ref="B266">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B265,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="267" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A267" s="8">
+        <f t="array" ref="A267">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A266,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B267" s="8">
+        <f t="array" ref="B267">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B266,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="268" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A268" s="8">
+        <f t="array" ref="A268">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A267,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B268" s="8">
+        <f t="array" ref="B268">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B267,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="269" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A269" s="8">
+        <f t="array" ref="A269">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A268,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B269" s="8">
+        <f t="array" ref="B269">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B268,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="270" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A270" s="8">
+        <f t="array" ref="A270">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A269,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B270" s="8">
+        <f t="array" ref="B270">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B269,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="271" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A271" s="8">
+        <f t="array" ref="A271">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A270,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B271" s="8">
+        <f t="array" ref="B271">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B270,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="272" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A272" s="8">
+        <f t="array" ref="A272">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A271,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B272" s="8">
+        <f t="array" ref="B272">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B271,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="273" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A273" s="8">
+        <f t="array" ref="A273">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A272,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B273" s="8">
+        <f t="array" ref="B273">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B272,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="274" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A274" s="8">
+        <f t="array" ref="A274">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A273,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B274" s="8">
+        <f t="array" ref="B274">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B273,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A275" s="8">
+        <f t="array" ref="A275">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A274,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B275" s="8">
+        <f t="array" ref="B275">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B274,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="276" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A276" s="8">
+        <f t="array" ref="A276">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A275,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B276" s="8">
+        <f t="array" ref="B276">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B275,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="277" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A277" s="8">
+        <f t="array" ref="A277">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A276,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B277" s="8">
+        <f t="array" ref="B277">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B276,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="278" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A278" s="8">
+        <f t="array" ref="A278">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A277,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B278" s="8">
+        <f t="array" ref="B278">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B277,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="279" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A279" s="8">
+        <f t="array" ref="A279">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A278,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B279" s="8">
+        <f t="array" ref="B279">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B278,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="280" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A280" s="8">
+        <f t="array" ref="A280">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A279,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B280" s="8">
+        <f t="array" ref="B280">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B279,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A281" s="8">
+        <f t="array" ref="A281">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A280,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B281" s="8">
+        <f t="array" ref="B281">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B280,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="282" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A282" s="8">
+        <f t="array" ref="A282">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A281,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B282" s="8">
+        <f t="array" ref="B282">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B281,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="283" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A283" s="8">
+        <f t="array" ref="A283">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A282,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B283" s="8">
+        <f t="array" ref="B283">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B282,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="284" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A284" s="8">
+        <f t="array" ref="A284">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A283,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B284" s="8">
+        <f t="array" ref="B284">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B283,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="285" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A285" s="8">
+        <f t="array" ref="A285">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A284,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B285" s="8">
+        <f t="array" ref="B285">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B284,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="286" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A286" s="8">
+        <f t="array" ref="A286">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A285,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B286" s="8">
+        <f t="array" ref="B286">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B285,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="287" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A287" s="8">
+        <f t="array" ref="A287">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A286,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B287" s="8">
+        <f t="array" ref="B287">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B286,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="288" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A288" s="8">
+        <f t="array" ref="A288">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A287,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B288" s="8">
+        <f t="array" ref="B288">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B287,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="289" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A289" s="8">
+        <f t="array" ref="A289">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A288,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B289" s="8">
+        <f t="array" ref="B289">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B288,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="290" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A290" s="8">
+        <f t="array" ref="A290">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A289,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B290" s="8">
+        <f t="array" ref="B290">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B289,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="291" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A291" s="8">
+        <f t="array" ref="A291">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A290,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B291" s="8">
+        <f t="array" ref="B291">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B290,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="292" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A292" s="8">
+        <f t="array" ref="A292">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A291,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B292" s="8">
+        <f t="array" ref="B292">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B291,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="293" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A293" s="8">
+        <f t="array" ref="A293">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A292,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B293" s="8">
+        <f t="array" ref="B293">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B292,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="294" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A294" s="8">
+        <f t="array" ref="A294">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A293,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B294" s="8">
+        <f t="array" ref="B294">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B293,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="295" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A295" s="8">
+        <f t="array" ref="A295">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A294,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B295" s="8">
+        <f t="array" ref="B295">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B294,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="296" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A296" s="8">
+        <f t="array" ref="A296">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A295,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B296" s="8">
+        <f t="array" ref="B296">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B295,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="297" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A297" s="8">
+        <f t="array" ref="A297">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A296,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B297" s="8">
+        <f t="array" ref="B297">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B296,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="298" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A298" s="8">
+        <f t="array" ref="A298">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A297,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B298" s="8">
+        <f t="array" ref="B298">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B297,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="299" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A299" s="8">
+        <f t="array" ref="A299">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A298,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B299" s="8">
+        <f t="array" ref="B299">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B298,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+    </row>
+    <row r="300" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A300" s="8">
+        <f t="array" ref="A300">IFERROR(INDEX(Materiales!$A$2:$A$300,MATCH(0,COUNTIF($A$1:A299,Materiales!$A$2:$A$300)+IF(Materiales!$A$2:$A$300="",1,0),0)),"")</f>
+      </c>
+      <c r="B300" s="8">
+        <f t="array" ref="B300">IFERROR(INDEX(Colecciones!$A$2:$A$300,MATCH(0,COUNTIF($B$1:B299,Colecciones!$A$2:$A$300)+IF(Colecciones!$A$2:$A$300="",1,0),0)),"")</f>
       </c>
     </row>
   </sheetData>

</xml_diff>